<commit_message>
Update arima model forecasts
</commit_message>
<xml_diff>
--- a/Evaluation/dm_test/dm_test_non_benchmark_models.xlsx
+++ b/Evaluation/dm_test/dm_test_non_benchmark_models.xlsx
@@ -470,10 +470,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-0.031</v>
+        <v>1.495</v>
       </c>
       <c r="E2" t="n">
-        <v>0.512</v>
+        <v>0.067</v>
       </c>
       <c r="F2" t="b">
         <v>0</v>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.733</v>
+        <v>3.875</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.793</v>
+        <v>4.131</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -648,10 +648,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-1.255</v>
+        <v>-0.616</v>
       </c>
       <c r="E8" t="n">
-        <v>0.895</v>
+        <v>0.731</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -675,10 +675,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3.154</v>
+        <v>2.683</v>
       </c>
       <c r="E9" t="n">
-        <v>0.001</v>
+        <v>0.004</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3.31</v>
+        <v>2.696</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -826,10 +826,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.934</v>
+        <v>1.829</v>
       </c>
       <c r="E14" t="n">
-        <v>0.027</v>
+        <v>0.034</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -857,10 +857,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.199</v>
+        <v>1.508</v>
       </c>
       <c r="E15" t="n">
-        <v>0.115</v>
+        <v>0.066</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
@@ -884,10 +884,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1.011</v>
+        <v>1.251</v>
       </c>
       <c r="E16" t="n">
-        <v>0.156</v>
+        <v>0.106</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
@@ -996,10 +996,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.141</v>
+        <v>0.671</v>
       </c>
       <c r="E20" t="n">
-        <v>0.444</v>
+        <v>0.251</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -1023,10 +1023,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-1.079</v>
+        <v>-1.06</v>
       </c>
       <c r="E21" t="n">
-        <v>0.86</v>
+        <v>0.855</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
@@ -1050,10 +1050,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.675</v>
+        <v>2.521</v>
       </c>
       <c r="E22" t="n">
-        <v>0.047</v>
+        <v>0.006</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -1162,10 +1162,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.868</v>
+        <v>1.574</v>
       </c>
       <c r="E26" t="n">
-        <v>0.193</v>
+        <v>0.058</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -1189,10 +1189,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.446</v>
+        <v>1.402</v>
       </c>
       <c r="E27" t="n">
-        <v>0.074</v>
+        <v>0.081</v>
       </c>
       <c r="F27" t="b">
         <v>0</v>
@@ -1216,10 +1216,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.347</v>
+        <v>1.558</v>
       </c>
       <c r="E28" t="n">
-        <v>0.089</v>
+        <v>0.06</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -1324,10 +1324,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.136</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>0.446</v>
+        <v>0.21</v>
       </c>
       <c r="F32" t="b">
         <v>0</v>
@@ -1351,15 +1351,19 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.735</v>
+        <v>1.816</v>
       </c>
       <c r="E33" t="n">
-        <v>0.231</v>
+        <v>0.035</v>
       </c>
       <c r="F33" t="b">
-        <v>0</v>
-      </c>
-      <c r="G33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>pls</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1378,10 +1382,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.995</v>
+        <v>2.961</v>
       </c>
       <c r="E34" t="n">
-        <v>0.023</v>
+        <v>0.002</v>
       </c>
       <c r="F34" t="b">
         <v>1</v>
@@ -1494,10 +1498,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.935</v>
+        <v>2.048</v>
       </c>
       <c r="E38" t="n">
-        <v>0.027</v>
+        <v>0.02</v>
       </c>
       <c r="F38" t="b">
         <v>1</v>
@@ -1525,15 +1529,19 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1.17</v>
+        <v>1.782</v>
       </c>
       <c r="E39" t="n">
-        <v>0.121</v>
+        <v>0.037</v>
       </c>
       <c r="F39" t="b">
-        <v>0</v>
-      </c>
-      <c r="G39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>pls</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1552,7 +1560,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2.88</v>
+        <v>2.865</v>
       </c>
       <c r="E40" t="n">
         <v>0.002</v>
@@ -1699,10 +1707,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>-0.393</v>
+        <v>0.734</v>
       </c>
       <c r="E45" t="n">
-        <v>0.653</v>
+        <v>0.232</v>
       </c>
       <c r="F45" t="b">
         <v>0</v>
@@ -1726,10 +1734,10 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.853</v>
+        <v>1.617</v>
       </c>
       <c r="E46" t="n">
-        <v>0.197</v>
+        <v>0.053</v>
       </c>
       <c r="F46" t="b">
         <v>0</v>
@@ -1842,10 +1850,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>-0.635</v>
+        <v>-0.384</v>
       </c>
       <c r="E50" t="n">
-        <v>0.737</v>
+        <v>0.65</v>
       </c>
       <c r="F50" t="b">
         <v>0</v>
@@ -1869,10 +1877,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>-1.177</v>
+        <v>0.493</v>
       </c>
       <c r="E51" t="n">
-        <v>0.88</v>
+        <v>0.311</v>
       </c>
       <c r="F51" t="b">
         <v>0</v>
@@ -1896,7 +1904,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2.624</v>
+        <v>2.655</v>
       </c>
       <c r="E52" t="n">
         <v>0.004</v>
@@ -2016,10 +2024,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>-1.7</v>
+        <v>-1.499</v>
       </c>
       <c r="E56" t="n">
-        <v>0.955</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="F56" t="b">
         <v>0</v>
@@ -2043,7 +2051,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>-4.044</v>
+        <v>-3.783</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
@@ -2070,10 +2078,10 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.186</v>
+        <v>0.917</v>
       </c>
       <c r="E58" t="n">
-        <v>0.426</v>
+        <v>0.18</v>
       </c>
       <c r="F58" t="b">
         <v>0</v>
@@ -2186,10 +2194,10 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.408</v>
+        <v>0.36</v>
       </c>
       <c r="E62" t="n">
-        <v>0.342</v>
+        <v>0.359</v>
       </c>
       <c r="F62" t="b">
         <v>0</v>
@@ -2213,19 +2221,15 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.822</v>
+        <v>1.167</v>
       </c>
       <c r="E63" t="n">
-        <v>0.034</v>
+        <v>0.122</v>
       </c>
       <c r="F63" t="b">
-        <v>1</v>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>pls</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2244,19 +2248,15 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2.466</v>
+        <v>1.358</v>
       </c>
       <c r="E64" t="n">
-        <v>0.007</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="F64" t="b">
-        <v>1</v>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>rf</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2360,10 +2360,10 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.477</v>
+        <v>1.379</v>
       </c>
       <c r="E68" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F68" t="b">
         <v>0</v>
@@ -2387,10 +2387,10 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>-2.197</v>
+        <v>0.137</v>
       </c>
       <c r="E69" t="n">
-        <v>0.986</v>
+        <v>0.446</v>
       </c>
       <c r="F69" t="b">
         <v>0</v>
@@ -2414,10 +2414,10 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>-0.343</v>
+        <v>1.452</v>
       </c>
       <c r="E70" t="n">
-        <v>0.634</v>
+        <v>0.073</v>
       </c>
       <c r="F70" t="b">
         <v>0</v>

</xml_diff>